<commit_message>
thay đổi mã lớp, tên lớp
</commit_message>
<xml_diff>
--- a/docs/demo/sinhvien_hop_le.xlsx
+++ b/docs/demo/sinhvien_hop_le.xlsx
@@ -38,7 +38,7 @@
     <x:t>Địa chỉ</x:t>
   </x:si>
   <x:si>
-    <x:t>Mã lớp</x:t>
+    <x:t>Lớp</x:t>
   </x:si>
   <x:si>
     <x:t>2001250101</x:t>
@@ -143,7 +143,7 @@
     <x:t>Ngày tạo:</x:t>
   </x:si>
   <x:si>
-    <x:t>28/10/2026 21:11</x:t>
+    <x:t>29/10/2026 18:51</x:t>
   </x:si>
   <x:si>
     <x:t>• Nhập dữ liệu ở sheet "DanhSach", mỗi sinh viên một dòng, giữ nguyên dòng tiêu đề cột.</x:t>
@@ -158,7 +158,7 @@
     <x:t>• Giới tính: Nam hoặc Nữ.  Email, SĐT (10 số, bắt đầu bằng 0), Địa chỉ: có thể để trống.</x:t>
   </x:si>
   <x:si>
-    <x:t>• Mã lớp: phải là lớp đã có (xem danh sách bên dưới).</x:t>
+    <x:t>• Lớp: ghi tên lớp đã có, ví dụ 16DHTH01 (xem danh sách bên dưới).</x:t>
   </x:si>
   <x:si>
     <x:t>• Tài khoản đăng nhập được tạo tự động: tên đăng nhập = MSSV, mật khẩu = ngày sinh ddMMyyyy.</x:t>
@@ -191,31 +191,28 @@
     <x:t>16DHTH01</x:t>
   </x:si>
   <x:si>
-    <x:t>Mã lớp hợp lệ:</x:t>
+    <x:t>Lớp hợp lệ:</x:t>
   </x:si>
   <x:si>
     <x:t>16DHATTT01</x:t>
   </x:si>
   <x:si>
-    <x:t>Đại học An toàn thông tin 16 - Lớp 01</x:t>
+    <x:t>An toàn thông tin – niên khóa 2025-2029</x:t>
   </x:si>
   <x:si>
     <x:t>16DHHTTT01</x:t>
   </x:si>
   <x:si>
-    <x:t>Đại học Hệ thống thông tin 16 - Lớp 01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Đại học Khoa học dữ liệu 16 - Lớp 01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Đại học Công nghệ thông tin 16 - Lớp 01</x:t>
+    <x:t>Hệ thống thông tin – niên khóa 2025-2029</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Khoa học dữ liệu – niên khóa 2025-2029</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Công nghệ thông tin – niên khóa 2025-2029</x:t>
   </x:si>
   <x:si>
     <x:t>16DHTH02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Đại học Công nghệ thông tin 16 - Lớp 02</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -6000,7 +5997,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>